<commit_message>
Updating elnino-app prob vals
</commit_message>
<xml_diff>
--- a/blog/elnino-app/prob_vals.xlsx
+++ b/blog/elnino-app/prob_vals.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\demersales1\Documents\LuisLauM.github.io\blog\elnino-app\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\indem\Documents\LuisLauM.github.io\blog\elnino-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F8D00EF-71EE-43B2-A3E8-BF571C9E36C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166EFA0C-B340-428D-A50D-0D397E77CCD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E84E93AA-1F6F-422A-B619-73DFFD9A6158}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E84E93AA-1F6F-422A-B619-73DFFD9A6158}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -451,13 +451,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{645C29F5-28DB-4A95-A3F0-2FC922850167}">
-  <dimension ref="A1:S87"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S90"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1"/>
       <c r="B1" s="5" t="s">
         <v>10</v>
@@ -482,7 +482,7 @@
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -541,7 +541,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>43966</v>
       </c>
@@ -564,7 +564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>43994</v>
       </c>
@@ -602,7 +602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>44025</v>
       </c>
@@ -640,7 +640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>44056</v>
       </c>
@@ -675,7 +675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>44092</v>
       </c>
@@ -707,7 +707,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>44123</v>
       </c>
@@ -742,7 +742,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>44141</v>
       </c>
@@ -777,7 +777,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>44176</v>
       </c>
@@ -806,7 +806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>44210</v>
       </c>
@@ -832,7 +832,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>44239</v>
       </c>
@@ -855,7 +855,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>44267</v>
       </c>
@@ -881,7 +881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>44301</v>
       </c>
@@ -907,7 +907,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>44330</v>
       </c>
@@ -930,7 +930,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>44358</v>
       </c>
@@ -953,7 +953,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>44389</v>
       </c>
@@ -976,7 +976,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>44421</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>44452</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>44483</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>44512</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>44545</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>44575</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>44606</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>44634</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>44664</v>
       </c>
@@ -1180,7 +1180,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>44694</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>44728</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>44757</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>44785</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>44819</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>44847</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>44879</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>44910</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>44939</v>
       </c>
@@ -1387,7 +1387,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>44973</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>45001</v>
       </c>
@@ -1427,7 +1427,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>45015</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>45029</v>
       </c>
@@ -1467,7 +1467,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>45044</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>45057</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>45077</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>45093</v>
       </c>
@@ -1541,7 +1541,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>45112</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>45128</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>45149</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>45169</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
         <v>45183</v>
       </c>
@@ -1650,7 +1650,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>45197</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
         <v>45212</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
         <v>45228</v>
       </c>
@@ -1719,7 +1719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
         <v>45240</v>
       </c>
@@ -1739,7 +1739,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
         <v>45254</v>
       </c>
@@ -1762,7 +1762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
         <v>45275</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
         <v>45289</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
         <v>45303</v>
       </c>
@@ -1831,7 +1831,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
         <v>45317</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
         <v>45338</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
         <v>45352</v>
       </c>
@@ -1909,7 +1909,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
         <v>45366</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
         <v>45387</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
         <v>45401</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
         <v>45429</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
         <v>45457</v>
       </c>
@@ -2033,7 +2033,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
         <v>45485</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
         <v>45520</v>
       </c>
@@ -2079,7 +2079,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
         <v>45548</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
         <v>45583</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
         <v>45614</v>
       </c>
@@ -2154,7 +2154,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
         <v>45639</v>
       </c>
@@ -2180,7 +2180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
         <v>45674</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
         <v>45702</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
         <v>45716</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
         <v>45730</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
         <v>45744</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
         <v>45763</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>45793</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
         <v>45821</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>45853</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
         <v>45884</v>
       </c>
@@ -2395,7 +2395,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
         <v>45916</v>
       </c>
@@ -2415,7 +2415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
         <v>45947</v>
       </c>
@@ -2435,7 +2435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
         <v>45979</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
         <v>46009</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
         <v>46037</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
         <v>46052</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
         <v>46066</v>
       </c>
@@ -2550,6 +2550,72 @@
       </c>
       <c r="Q87">
         <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A88" s="2">
+        <v>46080</v>
+      </c>
+      <c r="E88">
+        <v>5</v>
+      </c>
+      <c r="F88">
+        <v>83</v>
+      </c>
+      <c r="G88">
+        <v>12</v>
+      </c>
+      <c r="O88">
+        <v>4</v>
+      </c>
+      <c r="P88">
+        <v>51</v>
+      </c>
+      <c r="Q88">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A89" s="2">
+        <v>46094</v>
+      </c>
+      <c r="E89">
+        <v>1</v>
+      </c>
+      <c r="F89">
+        <v>88</v>
+      </c>
+      <c r="G89">
+        <v>11</v>
+      </c>
+      <c r="O89">
+        <v>10</v>
+      </c>
+      <c r="P89">
+        <v>63</v>
+      </c>
+      <c r="Q89">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A90" s="2">
+        <v>46108</v>
+      </c>
+      <c r="F90">
+        <v>75</v>
+      </c>
+      <c r="G90">
+        <v>25</v>
+      </c>
+      <c r="O90">
+        <v>8</v>
+      </c>
+      <c r="P90">
+        <v>60</v>
+      </c>
+      <c r="Q90">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>